<commit_message>
feat: enhance AddStudentDialog UI with icon, refined layout, and improved feedback handling
</commit_message>
<xml_diff>
--- a/Sessions/3rd Ferdous session 456.xlsx
+++ b/Sessions/3rd Ferdous session 456.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4601,6 +4601,47 @@
       </c>
       <c r="K97" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Unknown 1</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>11:49:09 PM</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>[11:49:09 PM] Manually added</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>